<commit_message>
Checking in v3.06 Installer Script and Files.
Added Example Test Project
Added Original myRIO FPGA shipping project.
</commit_message>
<xml_diff>
--- a/0__Documentation/pp_Processed_Files_List.xlsx
+++ b/0__Documentation/pp_Processed_Files_List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\____SCRATCH_PAD\2026_06_22__Make_myRIO_Merge_Install\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{FA26FFFC-8833-4C26-991F-0CB6015BC14B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5914CF52-C816-4740-8808-6B2456DA6EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16065" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{472D1C9A-19CF-4329-B322-717BB1CFD404}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{472D1C9A-19CF-4329-B322-717BB1CFD404}"/>
   </bookViews>
   <sheets>
     <sheet name="pp_Processed_List" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5235" uniqueCount="2152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5237" uniqueCount="2154">
   <si>
     <t>File List of R:\</t>
   </si>
@@ -6476,6 +6476,12 @@
   </si>
   <si>
     <t>R:\National Instruments - myRIO install additions\_Legal Information\NI-RIO 21.5 for LabVIEW Real-Time 21.50.49262 {1AD2063F-C124-460D-840D-CD43380237C4}</t>
+  </si>
+  <si>
+    <t>vi.lib\FPGAPlugInAG</t>
+  </si>
+  <si>
+    <t>*Added Missing Directory</t>
   </si>
 </sst>
 </file>
@@ -7464,7 +7470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC1CCCA4-BA9E-4823-840B-4194637B7FE3}">
-  <dimension ref="A1:D2588"/>
+  <dimension ref="A1:D2591"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
@@ -43682,6 +43688,16 @@
         <v>2151</v>
       </c>
     </row>
+    <row r="2590" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2590" s="1" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="2591" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2591" s="1" t="s">
+        <v>2152</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>